<commit_message>
Updated Openpyxl for report generation
</commit_message>
<xml_diff>
--- a/backend/temp/invoices_export.xlsx
+++ b/backend/temp/invoices_export.xlsx
@@ -423,14 +423,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
     <col width="29" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -465,12 +465,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Vendor/Exporter</t>
+          <t>Exporter (Vendor)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Customer/Importer</t>
+          <t>Importer (Customer)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -520,53 +520,109 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>14623</t>
+          <t>146989</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2025-01-01</t>
+          <t>2025-03-01</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Eurasia Trade Corp (Russia)</t>
+          <t>AstraZeneca (UK)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Eurasia Trade Corp (Russia)</t>
+          <t>MSC (INDIA)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>russia</t>
+          <t>india</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>266500</v>
       </c>
       <c r="I2" t="n">
+        <v>35525</v>
+      </c>
+      <c r="J2" t="n">
+        <v>13.33</v>
+      </c>
+      <c r="K2" t="n">
+        <v>302025</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>2026-03-02 17:42:03.695845</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>14623</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Dragon Global Exports Ltd (China)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Eurasia Trade Corp (Russia)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>russia</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>266500</v>
+      </c>
+      <c r="I3" t="n">
         <v>21395</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J3" t="n">
         <v>8.029999999999999</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K3" t="n">
         <v>287895</v>
       </c>
-      <c r="L2" t="n">
-        <v>25</v>
-      </c>
-      <c r="M2" t="inlineStr">
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>2026-03-02 03:51:45.672851</t>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-03-02 17:42:26.046520</t>
         </is>
       </c>
     </row>
@@ -581,7 +637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -657,7 +713,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14623</t>
+          <t>146989</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -695,14 +751,14 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>russia</t>
+          <t>india</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14623</t>
+          <t>146989</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -730,39 +786,39 @@
         <v>75000</v>
       </c>
       <c r="H3" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="I3" t="n">
-        <v>7500</v>
+        <v>18750</v>
       </c>
       <c r="J3" t="n">
-        <v>82500</v>
+        <v>93750</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>russia</t>
+          <t>india</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14623</t>
+          <t>146989</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Steel rod</t>
+          <t>Panadol tablets</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>720851</t>
+          <t>300490</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>steel_products</t>
+          <t>medicines</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -775,15 +831,150 @@
         <v>144000</v>
       </c>
       <c r="H4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I4" t="n">
+        <v>14400</v>
+      </c>
+      <c r="J4" t="n">
+        <v>158400</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>india</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>14623</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tron Ore Fines</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>260111</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>iron_ore</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>500</v>
+      </c>
+      <c r="F5" t="n">
+        <v>95</v>
+      </c>
+      <c r="G5" t="n">
+        <v>47500</v>
+      </c>
+      <c r="H5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2375</v>
+      </c>
+      <c r="J5" t="n">
+        <v>49875</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>russia</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>14623</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>hyundai venue</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>870321</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>passenger_cars</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G6" t="n">
+        <v>75000</v>
+      </c>
+      <c r="H6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" t="n">
+        <v>7500</v>
+      </c>
+      <c r="J6" t="n">
+        <v>82500</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>russia</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>14623</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Steel rod</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>720851</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>steel_products</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>200</v>
+      </c>
+      <c r="F7" t="n">
+        <v>720</v>
+      </c>
+      <c r="G7" t="n">
+        <v>144000</v>
+      </c>
+      <c r="H7" t="n">
         <v>8</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I7" t="n">
         <v>11520</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J7" t="n">
         <v>155520</v>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>russia</t>
         </is>

</xml_diff>